<commit_message>
Cargar resumen real y presupuesto de la reunión de Logística (24 ago)
Excel de Presupuesto de Logística poblado con 16 ítems reales de la
transcripción de la llamada (bus, radios, provisiones, vehículo de
carga, etc.). Resumen agregado a ministerio/CLAUDE.md, flagging la
discrepancia sin resolver entre la meta de 65 bolsas y el objetivo de
90 del inventario general. Tarea de resumen creada en ClickUp.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bow5YbwaecCKiNhDR9vvNU
</commit_message>
<xml_diff>
--- a/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
+++ b/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -502,6 +502,742 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ALQUILER BUS 55 PLAZAS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Empresa ya contactada (misma del reto anterior, nombre sin confirmar)</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>55 asientos, presupuesto con descuento negociado</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Urgente (presupuesto vence a los 15 días de recibido, 24 ago)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>~1.197€ (sin confirmar exacto, Marco lo dijo con dudas)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>A definir con Administración</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Correo con presupuesto ya recibido por Mariano, falta abrirlo y confirmar cifra exacta</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>RADIOS VHF GRAN ALCANCE (nuevas)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Por confirmar — Marco va a reconsultar a la empresa de radios</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Deben servir en montaña (10km+ con varias montañas de por medio), resistentes al agua — las alquiladas el reto anterior NO sirvieron</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Urgente, sin fecha exacta</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Marco le escribe a la empresa explicando que las anteriores no funcionaron</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ETIQUETAS/PEGATINAS DE PROVISIONES</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Proveedor de Julio (el más barato cotizado, tiene el link)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Paquete de 100</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Para pegar en las bolsas de provisiones armadas</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>~31,90€ (puede subir 2-3€ vs. la vez pasada)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Discrepancia sin resolver: faltan 39 según el plan de 65 bolsas nuevas, pero el inventario general pide 90 en total — no se resolvió en la llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BOLSAS VACÍAS PARA PROVISIONES</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Amazon (junto con bolsas de basura negras, para un solo pedido)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Paquete de 100</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Para armar las bolsas de provisiones nuevas</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Hay 34 actuales — comprar de más porque algunas vienen malas/no se pegan bien</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PALA METÁLICA PARA CARBÓN</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Amazon o Bricomart/Obramar (a definir)</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Para mover el carbón de la parrilla — la pala de la iglesia está destinada a otra cosa (agujero de la cruz)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Julio manda el link elegido para que Mariano arme el presupuesto</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CAÑAS PARA ANTORCHAS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Contacto de Jonathan (vía Marco Guanuchi)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1 paquete de 12</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Cañas de bambú para las antorchas — se corta a la mitad y se mete la antorcha</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Ya coordinado, se retira el domingo</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>~23-24€</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>A confirmar quién paga y si se reembolsa</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Resuelto (coordinación)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>YA COORDINADO — no hace falta el link de Amazon que había mandado el pastor, ese era para las antorchas en sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PLATOS CENA DEL REY (con logo grabado)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tedi</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Faltan 4 de las 52 necesarias (hay 48) — son de madera/tronquito</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>~12€ (no confirmado si es por unidad o total)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>David confirma stock real en la web de Tedi antes de comprar. Richard graba el nombre DESPUÉS de comprarlos, no antes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CINTA REFLECTANTE NOCTURNA PLATEADA</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Obramar o Leroy Merlin (a confirmar)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Material plástico gris que se ilumina de noche, para marcar el camino/rutas — NO es precinto normal</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>No se consiguió el reto anterior por buscarla a último momento</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ALARGADOR ELÉCTRICO</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Administración (Juliana)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Uno para el rótulo luminoso, otro alargador general</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Probar primero el alargador amarillo grande que ya tienen — puede no estar funcionando</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CAMIÓN CAJA ABIERTA / PICK-UP 4x4</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Por confirmar — un lugar en Valencia manda presupuesto el 25 ago</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Debe soportar 1.000kg. Mariano prefiere pick-up 4x4 (Ford Ranger/Hilux/Amarok/Isuzu) por sobre un camión largo tipo Iveco — más manejable en tramos difíciles de montaña</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Presupuesto llega el 25 ago a primera hora</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>David también evalúa opciones en Alicante/Castellón si en Valencia no aparece pick-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>FURGONETA (préstamo, no compra)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Jefferson</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Julio confirma con Jefferson si puede prestar furgoneta Y camión juntos — Mateo (dueño del otro camión posible) tiene el suyo con roturas frecuentes</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>No es compra, es préstamo — se incluye acá para no perder el seguimiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PEGATINA RUGE CON NOMBRE Y TALLA (impresa)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Levis</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Sin definir (por senderista)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Nombre + talla + logo Ruge, hecha en computadora/impresora (se descartó escribir a mano con rotulador)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sin definir, Julio consulta mañana 25 ago</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>A confirmar si entra en el mismo presupuesto que el rótulo luminoso</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Julio pide cotización y tiempos de entrega a Levis</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RÓTULO LUMINOSO INFERIOR "ESPAÑA"</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Levis</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Mismo ancho que el rótulo grande ya existente, más angosto en largo</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Sin definir, Julio consulta mañana 25 ago</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Marco Guanuchi manda fotos/video con las medidas del rótulo grande existente</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>FIGURAS PARA PREMIOS</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ya presupuestado por Marco Guanuchi (proveedor sin nombre dado)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Listo para enviar a Administración</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Ya definido (monto no dictado en la llamada)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Listo para enviar</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Mariano lo manda junto con otras cosas para no mandar de a una</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TRONCOS</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Contacto pendiente (Marco Jurado se lo pasa a Julio)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Para el reto — se recogen y Logística los lleva hasta el lugar</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Julio todavía no recibió el número de contacto</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AGUA PARA SENDERISTAS (garrafas)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Contacto de Adrián Rivera (equipo de Cocina), sin confirmar todavía</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Faltan 43 (de 90 necesarias, hay 157... revisar unidad, ver nota)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Deben ser garrafas iguales, mismo color y sabor que el reto anterior</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Adrián dijo que él se encarga y ya sabe dónde comprar, pero falta que confirme presupuesto/contacto real — Julio lo ve mañana 25 ago a las 15:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cruzar transcripción con las notas reales de Mariano y corregir el registro de Ruge
Resuelve la discrepancia 65 vs 90 bolsas de provisiones (65 es la
correcta), agrega detalle de la cuenta de Amazon de Ruge para la pala,
separa bolsas de basura en 100L/50L, separa los dos alargadores
eléctricos, y deja marcada sin resolver la contradicción sobre quién
contacta a Jonathan/Adrián Rivera (cañas/agua) — Mariano lo confirma.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bow5YbwaecCKiNhDR9vvNU
</commit_message>
<xml_diff>
--- a/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
+++ b/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -637,7 +637,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Discrepancia sin resolver: faltan 39 según el plan de 65 bolsas nuevas, pero el inventario general pide 90 en total — no se resolvió en la llamada</t>
+          <t>RESUELTO (nota real de Mariano en vivo): la meta correcta es 65 bolsas nuevas, no 90 — el 90 era del inventario viejo. Confirmado: hay 29 bolsas hechas, 34 bolsas vacías (comprar paquete de 100), 26 etiquetas (comprar 39, o sea un paquete de 100).</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Amazon o Bricomart/Obramar (a definir)</t>
+          <t>Amazon — cuenta específica de Ruge (no la personal de Julio)</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -729,7 +729,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Julio manda el link elegido para que Mariano arme el presupuesto</t>
+          <t>Julio le pasa el link a Mariano para comprar desde la cuenta de Amazon de Ruge — pedir factura al comprar (para Administración)</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>YA COORDINADO — no hace falta el link de Amazon que había mandado el pastor, ese era para las antorchas en sí</t>
+          <t>Contacto real: Jonathan (vía Marco Guanuchi según la llamada, pero la nota de asignación de tareas de Mariano dice que es David quien le pide a Jonathan — sin resolver quién lo hace finalmente). ~23-24€, ya coordinado, se retira el domingo</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Obramar o Leroy Merlin (a confirmar)</t>
+          <t>Obramat o Leroy Merlin (a confirmar)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1234,7 +1234,146 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Adrián dijo que él se encarga y ya sabe dónde comprar, pero falta que confirme presupuesto/contacto real — Julio lo ve mañana 25 ago a las 15:00</t>
+          <t>Corregido: es David quien tiene que pedirle el contacto/info a Adrián Rivera (según la asignación real de tareas de Mariano) — en la llamada se había dicho que Julio lo vería mañana 25 ago 15:00 si David no lograba contactarlo antes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BOLSAS DE BASURA NEGRAS 100L</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>A definir — Julio le pregunta a Marco dónde las compró la vez pasada</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Para tapar rótulos grandes (una sola flecha grande)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Julio repite la compra donde ya se compró antes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BOLSAS DE BASURA NEGRAS 50L</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>A definir — Julio le pregunta a Marco dónde las compró la vez pasada</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Para tapar rótulos normales/chicos (una sola flecha)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Julio repite la compra donde ya se compró antes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ALARGADOR ELÉCTRICO — LETRERO RUGE ILUMINADO</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Marcos Chiriguaya</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Distinto del alargador general (fila aparte) — específico para el letrero iluminado de Ruge</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>26 ago</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>A confirmar con Marcos Chiriguaya</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Julio se lo pide directo a Marcos Chiriguaya, no a Administración</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cruzar de verdad contra el inventario oficial de Marco Jurado
Corrige una afirmación previa incorrecta: la meta de 65 bolsas de
provisiones NO estaba resuelta contra el documento oficial, que sigue
en 90 — solo se había resuelto contra fuentes internas de Mariano.
También corrige gestión de la pala (Logística, no Administración) y
el alargador general (ya prestado por la iglesia, no hay que
comprarlo). Detecta 2 ítems ausentes del inventario oficial (teléfono
satelital, rótulo España) y uno nuevo no mencionado hoy (antorchas LED).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bow5YbwaecCKiNhDR9vvNU
</commit_message>
<xml_diff>
--- a/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
+++ b/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -590,7 +590,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Marco le escribe a la empresa explicando que las anteriores no funcionaron</t>
+          <t>Marco le escribe a la empresa explicando que las anteriores no funcionaron | Confirmado en el inventario oficial: reto=15 unidades, régimen=ALQUILADO.</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>RESUELTO (nota real de Mariano en vivo): la meta correcta es 65 bolsas nuevas, no 90 — el 90 era del inventario viejo. Confirmado: hay 29 bolsas hechas, 34 bolsas vacías (comprar paquete de 100), 26 etiquetas (comprar 39, o sea un paquete de 100).</t>
+          <t>⚠️ SIN RESOLVER DE VERDAD: en la llamada de hoy decidieron bajar la meta a 65 bolsas, pero el inventario OFICIAL de Marco Jurado (INVENTARIO_2026_RUGE_actualizado_21ago2026.xlsx) sigue diciendo reto=90, sin actualizar. Alguien tiene que avisarle a Marco Jurado del cambio a 65 para que lo corrija ahí — mientras tanto los dos documentos no coinciden.</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>NO — gestión es de Logística directamente, según el inventario oficial (no de Administración)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -836,10 +836,8 @@
           <t>Obramat o Leroy Merlin (a confirmar)</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Sin definir</t>
-        </is>
+      <c r="C9" t="n">
+        <v>2</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -880,7 +878,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Administración (Juliana)</t>
+          <t>YA ES PRESTADO por la Iglesia Impact Valencia (según inventario oficial) — no hay que comprarlo ni pedirlo a Juliana</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -908,12 +906,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>No aplica, ya está prestado</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Probar primero el alargador amarillo grande que ya tienen — puede no estar funcionando</t>
+          <t>Solo falta probar que funcione (el amarillo grande puede estar roto) — no es una gestión de compra</t>
         </is>
       </c>
     </row>
@@ -1374,6 +1372,145 @@
       <c r="I20" t="inlineStr">
         <is>
           <t>Julio se lo pide directo a Marcos Chiriguaya, no a Administración</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TELÉFONO SATELITAL</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>⚠️ NO aparece en el inventario oficial de Marco Jurado — se habló en la llamada pero no está cargado ahí. Confirmar con Marco Jurado si falta agregarlo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>RÓTULO LUMINOSO INFERIOR "ESPAÑA"</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Levis</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Mismo ancho que el rótulo grande existente, más angosto</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>⚠️ NO aparece en el inventario oficial</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Puede que Marco Jurado no lo haya cargado todavía — confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ANTORCHAS DE LED SOLARES</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Sin definir</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Faltan 6 (hay 24, reto 30)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ítem separado de las cañas — no se había incluido antes</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>26 ago (según reparto viejo)</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Detectado al cruzar con el inventario oficial — no se mencionó en la llamada de hoy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Armar minuta completa de la reunión de Logística y marcar ítems listos
Minuta con avances, compromisos por persona y fecha límite jueves 27
ago para todo lo que vencía en agosto. Marca en el excel de
presupuesto los 4 bloques que Mariano ya tiene presupuestados (bus,
premios, bolsas de provisiones + alimentos, antorchas) como listos
para mandar a Administración. Cargada también como comentario en
ClickUp.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bow5YbwaecCKiNhDR9vvNU
</commit_message>
<xml_diff>
--- a/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
+++ b/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
@@ -523,7 +523,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Urgente (presupuesto vence a los 15 días de recibido, 24 ago)</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>LISTO — Mariano ya tiene el presupuesto, falta enviarlo a Administración</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Urgente, sin fecha exacta</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sin definir</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>LISTO — Mariano ya tiene el presupuesto de bolsas + todo el contenido de alimentos, falta enviarlo a Administración. Pendiente</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sin definir</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>LISTO — Mariano ya tiene el presupuesto de bolsas + todo el contenido de alimentos, falta enviarlo a Administración. Pendiente</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sin definir</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Resuelto (coordinación)</t>
+          <t>LISTO — Mariano ya tiene el presupuesto, falta enviarlo a Administración</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sin definir</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sin definir</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sin definir</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Sin definir</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sin definir, Julio consulta mañana 25 ago</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sin definir, Julio consulta mañana 25 ago</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Listo para enviar</t>
+          <t>LISTO — Mariano ya tiene el presupuesto, falta enviarlo a Administración</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sin definir</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Sin definir</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>26 ago</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sin definir</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>26 ago (según reparto viejo)</t>
+          <t>Jueves 27 ago 2026</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">

</xml_diff>

<commit_message>
Carga presupuestos reales de Ruge (bus, camión, rótulo, figuras, alimentos)
Actualiza el excel de logística con los 4 presupuestos reales recibidos
hoy (camión Fandos Rent, rótulo VIS Publicidad, figuras 3D, listado de
alimentos para bolsas de provisiones) y los datos de los links de Amazon
pendientes de precio (bolsas, cinta reflectante, antorchas).
</commit_message>
<xml_diff>
--- a/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
+++ b/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Presupuesto Logística" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Presupuesto Logística" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -649,7 +649,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Amazon (junto con bolsas de basura negras, para un solo pedido)</t>
+          <t>Amazon — https://www.amazon.es/dp/B0CQ2CWX1Y</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente — no se pudo consultar el precio de Amazon desde este sistema (dominio bloqueado), confirmar precio con Mariano</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Hay 34 actuales — comprar de más porque algunas vienen malas/no se pegan bien</t>
+          <t>Hay 34 actuales — comprar de más porque algunas vienen malas/no se pegan bien. Necesitamos paquete de 100 (link de Amazon compartido 28 ago).</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Obramat o Leroy Merlin (a confirmar)</t>
+          <t>Amazon — https://www.amazon.es/dp/B0BHQDDXJ7</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -851,7 +851,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente — no se pudo consultar el precio de Amazon desde este sistema (dominio bloqueado), confirmar precio con Mariano</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>No se consiguió el reto anterior por buscarla a último momento</t>
+          <t>No se consiguió el reto anterior por buscarla a último momento. Link de Amazon compartido 28 ago 2026.</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Por confirmar — un lugar en Valencia manda presupuesto el 25 ago</t>
+          <t>Talleres Fandos S.L. (Fandos Rent) — sede Paterna, Valencia</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -931,32 +931,32 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Debe soportar 1.000kg. Mariano prefiere pick-up 4x4 (Ford Ranger/Hilux/Amarok/Isuzu) por sobre un camión largo tipo Iveco — más manejable en tramos difíciles de montaña</t>
+          <t>IVECO Daily caja abierta, 3 plazas, MMA 3.500kg, carga máx. ~1.000kg. Exteriores 6,87m largo. Zona carga 4,40m x 2,03m. 1.000km incluidos, 0,18€+IVA km extra. Depósito fianza 300€. Presupuesto Nº 0325/26.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Presupuesto llega el 25 ago a primera hora</t>
+          <t>Alquiler del 30/09/2026 11:00 al 05/10/2026</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>667,01€ IVA incluido</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Administración</t>
+          <t>Depósito 300€ + alquiler — forma de pago sin especificar en el presupuesto, confirmar con Fandos Rent (638 81 96 48)</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>LISTO — presupuesto real recibido, falta enviarlo a Administración</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>David también evalúa opciones en Alicante/Castellón si en Valencia no aparece pick-up</t>
+          <t>PDF de presupuesto real recibido 28 ago 2026, cargado en Drive. Válido 10 días desde el 25 ago (emisión) — revisar vencimiento si se demora la aprobación. Contacto: Pepito Pérez, 638 81 96 48.</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Levis</t>
+          <t>VIS Publicidad (+34 694 27 89 08)</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1068,32 +1068,32 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Mismo ancho que el rótulo grande ya existente, más angosto en largo</t>
+          <t>Vinilo con corte. El cliente (GOTIR/Ruge) envía el diseño.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Jueves 27 ago 2026</t>
+          <t>Sin fecha límite dada en el presupuesto</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>317,00€ sin IVA + IVA 21% (66,57€) = 383,57€ total</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>50% al aprobar + 50% en la entrega, efectivo o transferencia a ES89 2100 5513 4802 0022 3174 (Caixabank, a nombre de Levington Guerrero)</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>LISTO — presupuesto real recibido, falta enviarlo a Administración</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Marco Guanuchi manda fotos/video con las medidas del rótulo grande existente</t>
+          <t>PDF de presupuesto real recibido 28 ago 2026, cargado en Drive.</t>
         </is>
       </c>
     </row>
@@ -1105,25 +1105,25 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ya presupuestado por Marco Guanuchi (proveedor sin nombre dado)</t>
+          <t>Ya presupuestado por Marco Guanuchi (impresión 3D)</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Impresión 3D, 100mm por figura, material PLA (800g total para las 5), incluye posprocesado y pintado/acabado. 18€ por figura.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Listo para enviar a Administración</t>
+          <t>Sin fecha límite dada en el presupuesto</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Ya definido (monto no dictado en la llamada)</t>
+          <t>90,00€ (18€ x 5 figuras)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1133,12 +1133,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>LISTO — Mariano ya tiene el presupuesto, falta enviarlo a Administración</t>
+          <t>LISTO — presupuesto real recibido, falta enviarlo a Administración</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Mariano lo manda junto con otras cosas para no mandar de a una</t>
+          <t>⚠️ El inventario oficial de Marco Jurado pide 7 figuras (reto 50 hombres), este presupuesto es solo para 5 — confirmar con Mariano si faltan 2 más por cotizar o si el reto real bajó a 5. PDF cargado en Drive.</t>
         </is>
       </c>
     </row>
@@ -1425,45 +1425,47 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RÓTULO LUMINOSO INFERIOR "ESPAÑA"</t>
+          <t>RÓTULO LUMINOSO INFERIOR "ESPAÑA" (fila duplicada)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Levis</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>1</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Mismo ancho que el rótulo grande existente, más angosto</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Jueves 27 ago 2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>A confirmar</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>⚠️ NO aparece en el inventario oficial</t>
+          <t>Ver fila 14 — mismo ítem, presupuesto ya cargado ahí</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Puede que Marco Jurado no lo haya cargado todavía — confirmar</t>
+          <t>Fila duplicada del ítem de la fila 14, se deja vacía para no contar dos veces en el presupuesto total.</t>
         </is>
       </c>
     </row>
@@ -1475,12 +1477,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Sin definir</t>
+          <t>Amazon — https://www.amazon.es/dp/B0DS2GM9QR</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Faltan 6 (hay 24, reto 30)</t>
+          <t>6 (mínimo de compra del paquete — solo se necesitan 3, faltan 6 según inventario oficial)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1495,7 +1497,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente — no se pudo consultar el precio de Amazon desde este sistema (dominio bloqueado), confirmar precio con Mariano</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1510,7 +1512,54 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Detectado al cruzar con el inventario oficial — no se mencionó en la llamada de hoy</t>
+          <t>Detectado al cruzar con el inventario oficial (faltan 6 de 30, hay 24). Mariano solo necesita 3, pero el paquete de Amazon tiene mínimo 6 — coincide con el faltante real, se compran las 6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ALIMENTO PARA BOLSA DE PROVISIONES (contenido, 10 productos)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Listado de compra (documento generado a partir de nota manuscrita)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>65 bolsas x contenido de cada producto (ver detalle)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MINIS RELLENO: Caja 8 paquetes — 1,95€ | GALLETA MANZANA: Caja 8 paquetes — 1,65€ | GALLETA CHOCO BLANCO: Caja 6 paquetes — 1,30€ | BARRA FRUTO SECO: Caja 6 paquetes — 1,65€ | CARAMELO BLANCO: Bolsa 45 unidades — 1,60€ | COLA CAO: Caja 50 sobres — 19,99€ | SNICKERS: Bolsa 5 unidades — 4,25€ | SOBRES TANG: Caja 30 unidades — 0,79€/unidad | RIN TIN MARUCHAN: Paquete 5 packs — 1,99€ | ATÚN GIRASOL DIDI: Pack 4 unidades — 1,99€</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sin fecha límite dada en el listado</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Ver precio por producto en el detalle — falta sumar el total según cantidad real de bolsas (65)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>LISTO — listado real recibido, falta calcular el total y enviarlo a Administración</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Es el contenido que va DENTRO de cada bolsa de provisiones (fila 5 son las bolsas vacías). Documento recibido 28 ago 2026, cargado en Drive.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Carga precios reales de Amazon y links de Drive de Mariano
Suma los precios confirmados por Mariano (bolsas provisiones, cinta
reflectante, antorchas LED) y reemplaza las referencias de Drive por los
links reales de su carpeta ministerial para los 4 PDFs de presupuesto.
</commit_message>
<xml_diff>
--- a/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
+++ b/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
@@ -669,7 +669,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Pendiente — no se pudo consultar el precio de Amazon desde este sistema (dominio bloqueado), confirmar precio con Mariano</t>
+          <t>10,99€ (paquete de 100, 229x305mm, 0,11€/unidad) — marca NefLaca, vendedor Paper Print Mart</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Hay 34 actuales — comprar de más porque algunas vienen malas/no se pegan bien. Necesitamos paquete de 100 (link de Amazon compartido 28 ago).</t>
+          <t>Hay 34 actuales — comprar de más porque algunas vienen malas/no se pegan bien. Link: https://www.amazon.es/dp/B0CQ2CWX1Y — precio confirmado por Mariano (captura) 28 ago 2026.</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Pendiente — no se pudo consultar el precio de Amazon desde este sistema (dominio bloqueado), confirmar precio con Mariano</t>
+          <t>11,99€ (rollo 5cm x 10m) — marca YXSF</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>No se consiguió el reto anterior por buscarla a último momento. Link de Amazon compartido 28 ago 2026.</t>
+          <t>⚠️ El producto del link es AMARILLA FLUORESCENTE, no plateada como dice el nombre original del ítem — confirmar con Mariano si el color no importa o si hace falta buscar otra. Cantidad necesaria original: 2 — si son 2 rollos, total 23,98€. Link: https://www.amazon.es/dp/B0BHQDDXJ7 — precio confirmado por Mariano (captura) 28 ago 2026.</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>PDF de presupuesto real recibido 28 ago 2026, cargado en Drive. Válido 10 días desde el 25 ago (emisión) — revisar vencimiento si se demora la aprobación. Contacto: Pepito Pérez, 638 81 96 48.</t>
+          <t>PDF de presupuesto real recibido 28 ago 2026. Drive: https://drive.google.com/file/d/1wAsPjYeVI59B_aIMXqs-A4_4vj3f-t46/view?usp=drive_link. Válido 10 días desde el 25 ago (emisión) — revisar vencimiento si se demora la aprobación. Contacto: Pepito Pérez, 638 81 96 48.</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>PDF de presupuesto real recibido 28 ago 2026, cargado en Drive.</t>
+          <t>PDF de presupuesto real recibido 28 ago 2026. Drive: https://drive.google.com/file/d/1iK3L8s8NCgFfXymTNTYn1B94iH_TraiX/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>⚠️ El inventario oficial de Marco Jurado pide 7 figuras (reto 50 hombres), este presupuesto es solo para 5 — confirmar con Mariano si faltan 2 más por cotizar o si el reto real bajó a 5. PDF cargado en Drive.</t>
+          <t>⚠️ El inventario oficial de Marco Jurado pide 7 figuras (reto 50 hombres), este presupuesto es solo para 5 — confirmar con Mariano si faltan 2 más por cotizar o si el reto real bajó a 5. PDF de presupuesto real recibido 28 ago 2026. Drive: https://drive.google.com/file/d/1v1CwPe1KVW6PnS5_VsIPvtY9ueIjWAoZ/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1497,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Pendiente — no se pudo consultar el precio de Amazon desde este sistema (dominio bloqueado), confirmar precio con Mariano</t>
+          <t>23,99€ (pack de 6, 4,00€/unidad) — marca FIFlying, con cupón 15% disponible</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Detectado al cruzar con el inventario oficial (faltan 6 de 30, hay 24). Mariano solo necesita 3, pero el paquete de Amazon tiene mínimo 6 — coincide con el faltante real, se compran las 6.</t>
+          <t>Detectado al cruzar con el inventario oficial (faltan 6 de 30, hay 24). Mariano solo necesita 3, pero el paquete de Amazon tiene mínimo 6 — coincide con el faltante real, se compran las 6. Link: https://www.amazon.es/dp/B0DS2GM9QR — precio confirmado por Mariano (captura) 28 ago 2026. Hay cupón de 15% aplicable, revisar si baja el precio final.</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Es el contenido que va DENTRO de cada bolsa de provisiones (fila 5 son las bolsas vacías). Documento recibido 28 ago 2026, cargado en Drive.</t>
+          <t>Es el contenido que va DENTRO de cada bolsa de provisiones (fila 5 son las bolsas vacías). Documento recibido 28 ago 2026. Drive: https://drive.google.com/file/d/12TJiNe615jcy5EZkLY8JUfWSoKXg3XCx/view?usp=drive_link</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualiza presupuesto de logística Ruge con presupuestos reales
Bus (Autocares Azahar, 1.190€), camión caja abierta (Fandos Rent,
667,01€), rótulo luminoso (VIS Publicidad, 383,57€), agua (Distribuciones
Pascual, 54,45€), pegatina con nombre y talla (gratis, regalo de Levis),
bolsas/cinta/antorchas (Amazon, precios confirmados), y alimento para
bolsas de provisiones cruzado contra el inventario oficial de Marco
Jurado con cantidades faltantes por producto. Figuras para premios
revertido a pendiente (presupuesto era para 5, hacen falta 7).
</commit_message>
<xml_diff>
--- a/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
+++ b/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
@@ -510,7 +510,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Empresa ya contactada (misma del reto anterior, nombre sin confirmar)</t>
+          <t>Autocares Azahar S.L. — Lorena Castillo (964539073 / 626190593), Camí de la Travessa 3, 12540 Vila-real</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -518,17 +518,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>55 asientos, presupuesto con descuento negociado</t>
+          <t>Bus 55 plazas, servicio de ida y vuelta. 01 oct: salida desde Manises, traslado a Xodos. 04 oct: salida de Xodos, traslado a Manises.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Jueves 27 ago 2026</t>
+          <t>Jueves 27 ago 2026 (venció, pendiente confirmación con Administración)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>~1.197€ (sin confirmar exacto, Marco lo dijo con dudas)</t>
+          <t>1.190,00€ IVA incluido</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -538,12 +538,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>LISTO — Mariano ya tiene el presupuesto, falta enviarlo a Administración</t>
+          <t>LISTO — presupuesto real confirmado 28 ago 2026, falta enviarlo a Administración</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Correo con presupuesto ya recibido por Mariano, falta abrirlo y confirmar cifra exacta</t>
+          <t>Precio exacto confirmado 28 ago 2026 (antes se estimaba ~1.197€ "con dudas") — cifra real: 1.190,00€.</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Levis</t>
+          <t>Levis (mismo proveedor del rótulo luminoso)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Nombre + talla + logo Ruge, hecha en computadora/impresora (se descartó escribir a mano con rotulador)</t>
+          <t>Nombre + talla + logo Ruge, hecha en computadora/impresora</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1033,22 +1033,22 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>0€ — GRATIS, Levis lo regala por hacer el cartel/rótulo luminoso con ellos</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>A confirmar si entra en el mismo presupuesto que el rótulo luminoso</t>
+          <t>No aplica — no requiere pago</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>LISTO — confirmado 28 ago 2026, sin costo, no requiere autorización de Administración</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Julio pide cotización y tiempos de entrega a Levis</t>
+          <t>Confirmado por Mariano 28 ago 2026: es un regalo de Levis por encargarles el rótulo luminoso (fila 14), no un ítem de presupuesto aparte.</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>90,00€ (18€ x 5 figuras)</t>
+          <t>Pendiente — el presupuesto de 90€ era para 5 figuras, Mariano confirmó que hace falta pedir presupuesto nuevo por 7</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1133,12 +1133,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>LISTO — presupuesto real recibido, falta enviarlo a Administración</t>
+          <t>Pendiente — falta el presupuesto nuevo por 7 unidades antes de mandarlo a Administración</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>⚠️ El inventario oficial de Marco Jurado pide 7 figuras (reto 50 hombres), este presupuesto es solo para 5 — confirmar con Mariano si faltan 2 más por cotizar o si el reto real bajó a 5. PDF de presupuesto real recibido 28 ago 2026. Drive: https://drive.google.com/file/d/1v1CwPe1KVW6PnS5_VsIPvtY9ueIjWAoZ/view?usp=drive_link</t>
+          <t>Confirmado por Mariano 28 ago 2026: el inventario oficial pide 7 figuras, hay que volver a cotizar (el presupuesto de 90€/5 unidades ya no sirve tal cual). PDF del presupuesto viejo (5 unidades), como referencia de precio unitario (18€/figura): https://drive.google.com/file/d/1v1CwPe1KVW6PnS5_VsIPvtY9ueIjWAoZ/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -1197,17 +1197,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Contacto de Adrián Rivera (equipo de Cocina), sin confirmar todavía</t>
+          <t>Distribuciones Pascual (C/Carmen Herrero Penella 1-3-21, 46470 Catarroja)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Faltan 43 (de 90 necesarias, hay 157... revisar unidad, ver nota)</t>
+          <t>50 garrafas (necesarias: faltan 43 de 90, este presupuesto cubre el redondeo a 50)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Deben ser garrafas iguales, mismo color y sabor que el reto anterior</t>
+          <t>Agua 5L, marca "La Serreta". Presupuesto Nº 2500004.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1217,22 +1217,22 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>54,45€ total (49,50€ base + 10% dto. ya aplicado + IVA 10%: 4,95€) — 0,99€/unidad antes de IVA</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Administración</t>
+          <t>Administración — forma de pago/domiciliación no especificada en el presupuesto</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>LISTO — presupuesto real recibido 28 ago 2026, falta enviarlo a Administración</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Corregido: es David quien tiene que pedirle el contacto/info a Adrián Rivera (según la asignación real de tareas de Mariano) — en la llamada se había dicho que Julio lo vería mañana 25 ago 15:00 si David no lograba contactarlo antes</t>
+          <t>Presupuesto emitido 26 ago 2026, válido según vencimiento indicado (26/08/2026 — revisar si sigue vigente al momento de aprobar).</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1529,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>65 bolsas x contenido de cada producto (ver detalle)</t>
+          <t>Ver cantidades faltantes por producto en el detalle (cruzado contra inventario oficial)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MINIS RELLENO: Caja 8 paquetes — 1,95€ | GALLETA MANZANA: Caja 8 paquetes — 1,65€ | GALLETA CHOCO BLANCO: Caja 6 paquetes — 1,30€ | BARRA FRUTO SECO: Caja 6 paquetes — 1,65€ | CARAMELO BLANCO: Bolsa 45 unidades — 1,60€ | COLA CAO: Caja 50 sobres — 19,99€ | SNICKERS: Bolsa 5 unidades — 4,25€ | SOBRES TANG: Caja 30 unidades — 0,79€/unidad | RIN TIN MARUCHAN: Paquete 5 packs — 1,99€ | ATÚN GIRASOL DIDI: Pack 4 unidades — 1,99€</t>
+          <t>Cruzado 28 ago 2026 contra el inventario oficial de Marco Jurado (INVENTARIO_2026_RUGE_actualizado_21ago2026.xlsx), columnas Stock actual / Reto 50 hombres:
+- MINIS RELLENO: stock 20, reto 90, faltan 70 → comprar 9 cajas de 8 paq (72u) x 1,95€ = 17,55€
+- GALLETA MANZANA: stock 6, reto 90, faltan 84 → comprar 11 cajas de 8 paq (88u) x 1,65€ = 18,15€
+- GALLETA CHOCO BLANCO: stock 0, reto 90, faltan 90 → comprar 15 cajas de 6 paq (90u) x 1,30€ = 19,50€
+- BARRA FRUTO SECO: stock 42, reto 180 (¡ojo, este reto es 180, no 90!), faltan 138 → comprar 23 cajas de 6 paq (138u) x 1,65€ = 37,95€
+- CARAMELO BLANCO: ⚠️ no se pudo cruzar con certeza — el oficial tiene "CARAMELOS SURTIDOS" (stock 2 paquetes, reto 5 paquetes) pero el nombre y la unidad no coinciden con "bolsa 45 und" del listado — confirmar con Marco Jurado si es el mismo ítem
+- COLA CAO: stock 24, reto 90, faltan 66 sobres → comprar 2 cajas de 50 sobres (100u) x 19,99€ = 39,98€
+- SNICKERS: stock 7, reto 90, faltan 83 → comprar 17 bolsas de 5u (85u) x 4,25€ = 72,25€
+- SOBRES TANG: stock 10, reto 90, faltan 80 → comprar 3 cajas de 30u (90u) x 0,79€/u = 71,10€
+- RIN TIN MARUCHAN: stock 58, reto 180, faltan 122 → comprar 25 packs de 5 (125u) x 1,99€ = 49,75€
+- ATÚN GIRASOL DIDI: stock 32, reto 90, faltan 58 → comprar 15 packs de 4u (60u) x 1,99€ = 29,85€</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1544,7 +1554,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Ver precio por producto en el detalle — falta sumar el total según cantidad real de bolsas (65)</t>
+          <t>~356,08€ estimado (suma de las cantidades sugeridas arriba, sin contar CARAMELO BLANCO — sin resolver)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1554,12 +1564,12 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>LISTO — listado real recibido, falta calcular el total y enviarlo a Administración</t>
+          <t>LISTO — cruzado contra el inventario oficial 28 ago 2026, falta resolver CARAMELO BLANCO y enviar a Administración</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Es el contenido que va DENTRO de cada bolsa de provisiones (fila 5 son las bolsas vacías). Documento recibido 28 ago 2026. Drive: https://drive.google.com/file/d/12TJiNe615jcy5EZkLY8JUfWSoKXg3XCx/view?usp=drive_link</t>
+          <t>Es el contenido que va DENTRO de cada bolsa de provisiones (fila 5 son las bolsas vacías). Cantidades sugeridas en paquetes/cajas — Julio/Marco confirman si prefieren otro tamaño de compra. Drive: https://drive.google.com/file/d/12TJiNe615jcy5EZkLY8JUfWSoKXg3XCx/view?usp=drive_link</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualiza presupuesto logística Ruge con presupuestos reales y reparto por persona
Bus (Autocares Azahar, 1.190€), camión abierto (Fandos Rent, 667,01€),
rótulo luminoso (VIS Publicidad, 383,57€), agua (Distribuciones Pascual,
54,45€), pegatina con nombre y talla (gratis, regalo de Levis), y alimento
para bolsas de provisiones (cruzado contra inventario oficial, ~356€).
Corrige dueño de figuras para premios (Marco G, cotización nueva por 7),
aclara troncos en curso (Julio ya contactando) y radios VHF/teléfono
satelital esperando número de Juliana.
</commit_message>
<xml_diff>
--- a/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
+++ b/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
@@ -585,12 +585,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente — Marco espera que Juliana le pase el número de contacto de la empresa (misma que teléfono satelital)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Marco le escribe a la empresa explicando que las anteriores no funcionaron | Confirmado en el inventario oficial: reto=15 unidades, régimen=ALQUILADO.</t>
+          <t>Marco le escribe a la empresa explicando que las anteriores no funcionaron | Confirmado en el inventario oficial: reto=15 unidades, régimen=ALQUILADO. ⚠️ 28 ago 2026: Marco está esperando que Juliana le mande el número de contacto — hay que recordarle a Marco que se lo pida.</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>⚠️ SIN RESOLVER DE VERDAD: en la llamada de hoy decidieron bajar la meta a 65 bolsas, pero el inventario OFICIAL de Marco Jurado (INVENTARIO_2026_RUGE_actualizado_21ago2026.xlsx) sigue diciendo reto=90, sin actualizar. Alguien tiene que avisarle a Marco Jurado del cambio a 65 para que lo corrija ahí — mientras tanto los dos documentos no coinciden.</t>
+          <t>Aclarado 28 ago 2026 por Mariano: hacen falta 90 en total (coincide con el inventario oficial), pero ya tenemos algunas en stock — por eso la cifra de compra rondaba los 65, no es una discrepancia real entre documentos.</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Faltan 4 de las 52 necesarias (hay 48) — son de madera/tronquito</t>
+          <t>Son de madera/tronquito. Aclarado 28 ago 2026: son TODOS los platos que faltan (no solo 4) — falta confirmar la cantidad exacta con Marcos Chiriguaya.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>David confirma stock real en la web de Tedi antes de comprar. Richard graba el nombre DESPUÉS de comprarlos, no antes</t>
+          <t>Aclarado 28 ago 2026: David tiene que confirmar precio y disponibilidad directo con Marcos Chiriguaya (no directo con Tedi). Richard graba el nombre DESPUÉS de comprarlos, no antes.</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ya presupuestado por Marco Guanuchi (impresión 3D)</t>
+          <t>Marco Guanuchi (pendiente de él, no de Julio) — presupuesto anterior de 5 unidades como referencia</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Confirmado por Mariano 28 ago 2026: el inventario oficial pide 7 figuras, hay que volver a cotizar (el presupuesto de 90€/5 unidades ya no sirve tal cual). PDF del presupuesto viejo (5 unidades), como referencia de precio unitario (18€/figura): https://drive.google.com/file/d/1v1CwPe1KVW6PnS5_VsIPvtY9ueIjWAoZ/view?usp=drive_link</t>
+          <t>Confirmado por Mariano 28 ago 2026: el inventario oficial pide 7 figuras y este pendiente es de Marco Guanuchi. Hay que volver a cotizar (el presupuesto de 90€/5 unidades ya no sirve tal cual, queda como referencia de precio: 18€/figura). PDF viejo: https://drive.google.com/file/d/1v1CwPe1KVW6PnS5_VsIPvtY9ueIjWAoZ/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -1180,12 +1180,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>EN CURSO — Marco Jurado ya le pasó el número de contacto a Julio, que ya está contactando</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Julio todavía no recibió el número de contacto</t>
+          <t>Actualizado 28 ago 2026: Marco Jurado ya le pasó el contacto a Julio y Julio ya lo está contactando — ya no está bloqueado esperando el número.</t>
         </is>
       </c>
     </row>
@@ -1383,42 +1383,42 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>Misma empresa que las radios VHF (fila 3)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pendiente — Marco espera el número de contacto de Juliana, mismo caso que las radios VHF</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>⚠️ NO aparece en el inventario oficial de Marco Jurado — se habló en la llamada pero no está cargado ahí. Confirmar con Marco Jurado si falta agregarlo.</t>
+          <t>⚠️ NO aparece en el inventario oficial de Marco Jurado — se habló en la llamada pero no está cargado ahí. Confirmar con Marco Jurado si falta agregarlo. 28 ago 2026: es la misma empresa de las radios VHF — Marco espera que Juliana le pase el número.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige comisión responsable de bolsas de basura, alargador y pala
Cruzado contra la columna "Comisión de revisión" del inventario oficial
de Marco Jurado: bolsas de basura 100L/50L y el alargador del letrero son
LOGÍSTICA Y EVENTOS (Eventos ejecuta, Logística corrobora) — reasignados
de Julio a Eventos. La pala metálica figura como COCINA, no Logística,
contradiciendo lo registrado en la llamada del 24 ago — queda marcada
para confirmar con Marco Jurado antes de asignarla.
</commit_message>
<xml_diff>
--- a/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
+++ b/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
@@ -729,7 +729,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Julio le pasa el link a Mariano para comprar desde la cuenta de Amazon de Ruge — pedir factura al comprar (para Administración)</t>
+          <t>⚠️ 28 ago 2026: el inventario oficial de Marco Jurado dice que la comisión de revisión es COCINA, no Logística — contradice lo registrado en la llamada del 24 ago ("gestión es de Logística directamente"). Confirmar con Marco Jurado cuál es la correcta antes de asignarlo a alguien.</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Actualizado 28 ago 2026: Marco Jurado ya le pasó el contacto a Julio y Julio ya lo está contactando — ya no está bloqueado esperando el número.</t>
+          <t>Actualizado 28 ago 2026: Marco Jurado ya le pasó el contacto a Julio y Julio ya lo está contactando — ya no está bloqueado esperando el número. ⚠️ Nota: la comisión de revisión oficial es LOGÍSTICA Y EVENTOS (Eventos debería ejecutar), pero como Julio ya arrancó la gestión en la práctica, se deja con él en vez de redirigir a mitad de camino.</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Julio repite la compra donde ya se compró antes</t>
+          <t>⚠️ 28 ago 2026: comisión de revisión oficial es LOGÍSTICA Y EVENTOS — según la regla ya confirmada por Marco Jurado, la segunda comisión (Eventos, Mauricio/Cristian) es quien gestiona/ejecuta, Logística solo corrobora. Reasignado de Julio a Eventos.</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Julio repite la compra donde ya se compró antes</t>
+          <t>⚠️ 28 ago 2026: comisión de revisión oficial es LOGÍSTICA Y EVENTOS — según la regla ya confirmada por Marco Jurado, la segunda comisión (Eventos, Mauricio/Cristian) es quien gestiona/ejecuta, Logística solo corrobora. Reasignado de Julio a Eventos.</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Julio se lo pide directo a Marcos Chiriguaya, no a Administración</t>
+          <t>⚠️ 28 ago 2026: comisión de revisión oficial es LOGÍSTICA Y EVENTOS — Eventos (Mauricio/Cristian) gestiona/ejecuta, Julio solo corrobora. Reasignado de Julio a Eventos.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualiza presupuesto de figuras para premios (7 unidades, 91€)
Cotización real recibida: 13€/figura x 7 = 91€, más barata por unidad
que la anterior (18€/figura x 5). Responsable: Marco Guanuchi.
</commit_message>
<xml_diff>
--- a/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
+++ b/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
@@ -1105,7 +1105,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Marco Guanuchi (pendiente de él, no de Julio) — presupuesto anterior de 5 unidades como referencia</t>
+          <t>Marco Guanuchi (impresión 3D)</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Pendiente — el presupuesto de 90€ era para 5 figuras, Mariano confirmó que hace falta pedir presupuesto nuevo por 7</t>
+          <t>91,00€ (13,00€ x 7 figuras)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1133,12 +1133,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Pendiente — falta el presupuesto nuevo por 7 unidades antes de mandarlo a Administración</t>
+          <t>LISTO — presupuesto real por 7 unidades recibido 28 ago 2026, falta enviarlo a Administración</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Confirmado por Mariano 28 ago 2026: el inventario oficial pide 7 figuras y este pendiente es de Marco Guanuchi. Hay que volver a cotizar (el presupuesto de 90€/5 unidades ya no sirve tal cual, queda como referencia de precio: 18€/figura). PDF viejo: https://drive.google.com/file/d/1v1CwPe1KVW6PnS5_VsIPvtY9ueIjWAoZ/view?usp=drive_link</t>
+          <t>Confirmado: cotización nueva por 7 unidades, más barata por unidad que la de 5 (13€ vs 18€/figura). Falta que Mariano suba el PDF a su Drive y pase el link.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualiza estado de platos Cena del Rey — casi resuelto
David ya consiguió y grabó los platos que faltaban, solo queda pendiente
que envíen la factura.
</commit_message>
<xml_diff>
--- a/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
+++ b/mariano-os/areas/ministerio/recursos/Presupuesto_Logistica_Ruge_24ago2026.xlsx
@@ -816,12 +816,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>CASI LISTO — David ya consiguió y grabó los platos que faltaban, solo falta que envíen la factura</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Aclarado 28 ago 2026: David tiene que confirmar precio y disponibilidad directo con Marcos Chiriguaya (no directo con Tedi). Richard graba el nombre DESPUÉS de comprarlos, no antes.</t>
+          <t>Actualizado 28 ago 2026: David ya consiguió los platos que faltaban y ya están grabados con "RUGE". Queda pendiente únicamente que envíen la factura de esos platos.</t>
         </is>
       </c>
     </row>

</xml_diff>